<commit_message>
docs: split scan and maintenance rules; update matrix and coverage
</commit_message>
<xml_diff>
--- a/templates/platform-coverage.xlsx
+++ b/templates/platform-coverage.xlsx
@@ -49,10 +49,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -419,62 +422,73 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>检索日期</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>平台</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>查询词</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>检索位/查询词</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>城市</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>检索日期</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>结果数</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>检索状态</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>相关候选数</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>入库数</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>访问限制</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>访问限制/筛选说明</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>证据链接</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="检索状态不合法" error="只允许：已检索 / 受限 / 未执行" type="list">
+      <formula1>"已检索,受限,未执行"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>